<commit_message>
Update supplementary materials and analytical files for published manuscript
</commit_message>
<xml_diff>
--- a/aLBI/aLBI Output.xlsx
+++ b/aLBI/aLBI Output.xlsx
@@ -1,75 +1,82 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project Work\Saheen sir\Nirjhor 18-19\Data Analysis\aLBI\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9703036D-5999-4CD0-B5F2-C872CAAB8825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Length_Parameters" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Froese_Indicators" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Target_vs_Catch" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Length_Parameters" sheetId="1" r:id="rId1"/>
+    <sheet name="Froese_Indicators" sheetId="2" r:id="rId2"/>
+    <sheet name="Target_vs_Catch" sheetId="3" r:id="rId3"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
-  <si>
-    <t xml:space="preserve">Parameters</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean_estimate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lower_CI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Upper_CI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lmax</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Linf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lmat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lopt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lopt_p10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lopt_m10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mean_froese</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pmat</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Popt</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pmega</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Froese_catch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Froese_tar</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
+  <si>
+    <t>Parameters</t>
+  </si>
+  <si>
+    <t>Mean_estimate</t>
+  </si>
+  <si>
+    <t>Lower_CI</t>
+  </si>
+  <si>
+    <t>Upper_CI</t>
+  </si>
+  <si>
+    <t>Lmax</t>
+  </si>
+  <si>
+    <t>Linf</t>
+  </si>
+  <si>
+    <t>Lmat</t>
+  </si>
+  <si>
+    <t>Lopt</t>
+  </si>
+  <si>
+    <t>Lopt_p10</t>
+  </si>
+  <si>
+    <t>Lopt_m10</t>
+  </si>
+  <si>
+    <t>Mean_froese</t>
+  </si>
+  <si>
+    <t>Pmat</t>
+  </si>
+  <si>
+    <t>Popt</t>
+  </si>
+  <si>
+    <t>Pmega</t>
+  </si>
+  <si>
+    <t>Froese_catch</t>
+  </si>
+  <si>
+    <t>Froese_tar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -98,13 +105,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -386,11 +405,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -404,102 +423,102 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="n">
-        <v>34.5016380379956</v>
-      </c>
-      <c r="C2" t="n">
-        <v>33.5536788827177</v>
-      </c>
-      <c r="D2" t="n">
-        <v>35.3672854998113</v>
-      </c>
-    </row>
-    <row r="3">
+      <c r="B2">
+        <v>34.501638037995598</v>
+      </c>
+      <c r="C2">
+        <v>33.553678882717698</v>
+      </c>
+      <c r="D2">
+        <v>35.367285499811302</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" t="n">
-        <v>36.3175137242059</v>
-      </c>
-      <c r="C3" t="n">
-        <v>35.3196619818081</v>
-      </c>
-      <c r="D3" t="n">
-        <v>37.2287215787487</v>
-      </c>
-    </row>
-    <row r="4">
+      <c r="B3">
+        <v>36.317513724205902</v>
+      </c>
+      <c r="C3">
+        <v>35.319661981808103</v>
+      </c>
+      <c r="D3">
+        <v>37.228721578748697</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="n">
-        <v>21.0363031557507</v>
-      </c>
-      <c r="C4" t="n">
-        <v>20.0743137982584</v>
-      </c>
-      <c r="D4" t="n">
-        <v>21.992472433666</v>
-      </c>
-    </row>
-    <row r="5">
+      <c r="B4">
+        <v>21.036303155750701</v>
+      </c>
+      <c r="C4">
+        <v>20.074313798258402</v>
+      </c>
+      <c r="D4">
+        <v>21.992472433665998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
-      <c r="B5" t="n">
-        <v>21.7172851936536</v>
-      </c>
-      <c r="C5" t="n">
-        <v>20.0322895793874</v>
-      </c>
-      <c r="D5" t="n">
+      <c r="B5">
+        <v>21.717285193653598</v>
+      </c>
+      <c r="C5">
+        <v>20.032289579387399</v>
+      </c>
+      <c r="D5">
         <v>23.55706979899</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="n">
-        <v>23.889013713019</v>
-      </c>
-      <c r="C6" t="n">
-        <v>22.0355185373262</v>
-      </c>
-      <c r="D6" t="n">
+      <c r="B6">
+        <v>23.889013713019001</v>
+      </c>
+      <c r="C6">
+        <v>22.035518537326201</v>
+      </c>
+      <c r="D6">
         <v>25.912776778889</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" t="n">
+      <c r="B7">
         <v>19.5455566742882</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>18.0290606214487</v>
       </c>
-      <c r="D7" t="n">
-        <v>21.201362819091</v>
+      <c r="D7">
+        <v>21.201362819090999</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -513,60 +532,60 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="n">
-        <v>65.0313286024618</v>
-      </c>
-      <c r="C2" t="n">
-        <v>58.4346602031108</v>
-      </c>
-      <c r="D2" t="n">
-        <v>70.8962976274279</v>
-      </c>
-    </row>
-    <row r="3">
+      <c r="B2" s="1">
+        <v>65.031328602461798</v>
+      </c>
+      <c r="C2" s="1">
+        <v>58.434660203110802</v>
+      </c>
+      <c r="D2" s="1">
+        <v>70.896297627427899</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="n">
-        <v>42.4940777436779</v>
-      </c>
-      <c r="C3" t="n">
-        <v>30.9827920451477</v>
-      </c>
-      <c r="D3" t="n">
-        <v>54.081134352719</v>
-      </c>
-    </row>
-    <row r="4">
+      <c r="B3" s="1">
+        <v>42.494077743677899</v>
+      </c>
+      <c r="C3" s="1">
+        <v>30.982792045147701</v>
+      </c>
+      <c r="D3" s="1">
+        <v>54.081134352718998</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="n">
-        <v>31.783523501758</v>
-      </c>
-      <c r="C4" t="n">
-        <v>14.0264415529798</v>
-      </c>
-      <c r="D4" t="n">
-        <v>52.3830530885006</v>
+      <c r="B4" s="1">
+        <v>31.783523501758001</v>
+      </c>
+      <c r="C4" s="1">
+        <v>14.026441552979801</v>
+      </c>
+      <c r="D4" s="1">
+        <v>52.383053088500603</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -577,41 +596,41 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" t="n">
-        <v>65.0313286024618</v>
-      </c>
-      <c r="C2" t="n">
+      <c r="B2">
+        <v>65.031328602461798</v>
+      </c>
+      <c r="C2">
         <v>100</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="n">
-        <v>42.4940777436779</v>
-      </c>
-      <c r="C3" t="n">
+      <c r="B3">
+        <v>42.494077743677899</v>
+      </c>
+      <c r="C3">
         <v>100</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="n">
-        <v>31.783523501758</v>
-      </c>
-      <c r="C4" t="n">
+      <c r="B4">
+        <v>31.783523501758001</v>
+      </c>
+      <c r="C4">
         <v>20</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>